<commit_message>
feat(marketing): improve campaign materials and mobile capture
</commit_message>
<xml_diff>
--- a/public/downloads/lead-magnets/calculadora-ticket-medio.xlsx
+++ b/public/downloads/lead-magnets/calculadora-ticket-medio.xlsx
@@ -8,14 +8,16 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="600" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Leia primeiro" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Calculadora" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Comece aqui" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Painel rápido" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Calculadora" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">Calculadora!$A$1:$E$37</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Calculadora!$A$1:$E$37</definedName>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Leia primeiro'!$A$1:$F$16</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Calculadora!A1:E37</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">Calculadora!$A$1:$E$37</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Calculadora!$A$1:$E$37</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Comece aqui'!$A$1:$F$19</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Painel rápido'!$A$1:$I$18</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Calculadora!A1:E37</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,9 +29,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
-  <si>
-    <t xml:space="preserve">MATERIAL PRÁTICO FLOWO</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="58">
+  <si>
+    <t xml:space="preserve">FLOWO · MATERIAL PRÁTICO</t>
   </si>
   <si>
     <t xml:space="preserve">Calculadora de ticket médio</t>
@@ -38,19 +40,46 @@
     <t xml:space="preserve">Entenda quanto cada atendimento gera em média e quais serviços formam o faturamento.</t>
   </si>
   <si>
-    <t xml:space="preserve">flowo.com.br</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COMO USAR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. Informe quantidade e preço médio por serviço.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Informe o número total de atendimentos únicos do período.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Compare ticket atual e meta sem confundir faturamento com lucro.</t>
+    <t xml:space="preserve">Veja o resumo na próxima aba. Depois, preencha somente as células rosadas e volte ao resumo para decidir o que fazer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informe quantidade e preço médio por serviço.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Informe o número total de atendimentos únicos do período.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compare ticket atual e meta sem confundir faturamento com lucro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LEGENDA RÁPIDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIGITE AQUI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESULTADO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ATENÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Células rosadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Células verdes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Células amarelas</t>
   </si>
   <si>
     <t xml:space="preserve">ANTES DE COMEÇAR</t>
@@ -66,6 +95,54 @@
   </si>
   <si>
     <t xml:space="preserve">Material educativo. Adapte à realidade da sua barbearia e valide decisões contábeis, fiscais, trabalhistas e jurídicas com profissionais habilitados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flowo.com.br/recursos/materiais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FLOWO · RESUMO SIMPLES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quanto cada atendimento deixa no caixa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Veja o ticket atual, compare com a meta e escolha um serviço para trabalhar primeiro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TICKET ATUAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">META DE TICKET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALTA POR ATENDIMENTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">faturamento ÷ atendimentos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor definido por você</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diferença para a meta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRÓXIMA AÇÃO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escolha um serviço complementar real e calcule quantos clientes precisam aceitá-lo para reduzir a diferença.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMO LER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Preencha as células rosadas nas outras abas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Volte aqui para conferir os números principais.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Resolva primeiro o que estiver pendente ou bloqueado.</t>
   </si>
   <si>
     <t xml:space="preserve">Serviço</t>
@@ -137,7 +214,7 @@
     <numFmt numFmtId="165" formatCode="&quot;R$ &quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="21">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -170,15 +247,23 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="20"/>
+      <sz val="22"/>
       <color rgb="FF171810"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color rgb="FF6D6A61"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF6D6A61"/>
+      <color rgb="FF171810"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
@@ -201,13 +286,89 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF171810"/>
+      <color rgb="FF7A173F"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF1F7A50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FFA45D13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF6D6A61"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF171810"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFC52663"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF6D6A61"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="22"/>
+      <color rgb="FF1F7A50"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <color rgb="FFA45D13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF171810"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF7A173F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -223,12 +384,30 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF4F0E5"/>
-        <bgColor rgb="FFFBF9F3"/>
+        <bgColor rgb="FFFAEEDB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFBF9F3"/>
+        <bgColor rgb="FFF4F0E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8E9EF"/>
+        <bgColor rgb="FFF4F0E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7F3EC"/>
+        <bgColor rgb="FFF4F0E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFAEEDB"/>
         <bgColor rgb="FFF4F0E5"/>
       </patternFill>
     </fill>
@@ -282,7 +461,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -299,63 +478,107 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -368,7 +591,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -388,7 +611,31 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFF8E9EF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFBF9F3"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF7A173F"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE7F3EC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -409,14 +656,14 @@
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF1F7A50"/>
       <rgbColor rgb="FFD9D3C6"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF4F0E5"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFC52663"/>
+      <rgbColor rgb="FFFAEEDB"/>
+      <rgbColor rgb="FFE7F3EC"/>
+      <rgbColor rgb="FF7A173F"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFCCCCFF"/>
@@ -429,8 +676,8 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFF8E9EF"/>
+      <rgbColor rgb="FFF4F0E5"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
@@ -448,7 +695,7 @@
       <rgbColor rgb="FF339966"/>
       <rgbColor rgb="FF171810"/>
       <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FFA45D13"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
@@ -638,14 +885,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="18.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="1" style="0" width="18.83"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -655,7 +901,7 @@
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
     </row>
-    <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="40" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -665,7 +911,7 @@
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -676,147 +922,178 @@
       <c r="F3" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="10" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-    </row>
-    <row r="6" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B4" s="4"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4"/>
+    </row>
+    <row r="5" customFormat="false" ht="8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
+      <c r="C6" s="5" t="s">
+        <v>5</v>
+      </c>
       <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="E6" s="5" t="s">
+        <v>6</v>
+      </c>
       <c r="F6" s="5"/>
     </row>
-    <row r="7" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
+      <c r="C7" s="6" t="s">
+        <v>8</v>
+      </c>
       <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
+      <c r="E7" s="6" t="s">
+        <v>9</v>
+      </c>
       <c r="F7" s="6"/>
     </row>
-    <row r="8" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-    </row>
+    <row r="8" customFormat="false" ht="8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="9" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="10" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
-      <c r="F11" s="5"/>
-    </row>
-    <row r="12" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-    </row>
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1"/>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="8"/>
+      <c r="E10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="9"/>
+    </row>
+    <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="8"/>
+      <c r="E11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="9"/>
+    </row>
+    <row r="12" customFormat="false" ht="8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="13" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-    </row>
-    <row r="14" customFormat="false" ht="10" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-    </row>
-    <row r="15" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-    </row>
-    <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="6"/>
+      <c r="A13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="11"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+    </row>
+    <row r="17" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="46" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+    </row>
+    <row r="19" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="24">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A7:F7"/>
-    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
     <mergeCell ref="A9:F9"/>
-    <mergeCell ref="A10:F10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="E11:F11"/>
     <mergeCell ref="A13:F13"/>
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A15:F15"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A19:F19"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.511811023622047" footer="0.511811023622047"/>
@@ -833,6 +1110,224 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="A1:I17"/>
+  <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="1" style="0" width="14.84"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" customFormat="false" ht="40" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="5" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="44" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="n">
+        <f aca="false">Calculadora!$D$34</f>
+        <v>77.1785714285714</v>
+      </c>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15" t="n">
+        <f aca="false">Calculadora!$D$35</f>
+        <v>75</v>
+      </c>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15" t="n">
+        <f aca="false">Calculadora!$D$36</f>
+        <v>-2.17857142857143</v>
+      </c>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+    </row>
+    <row r="7" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16"/>
+      <c r="D7" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="26" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
+        <v>34</v>
+      </c>
+      <c r="B14" s="18"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+    </row>
+    <row r="15" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+    </row>
+    <row r="17" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+    </row>
+  </sheetData>
+  <mergeCells count="18">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="A10:I10"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="A14:I14"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A17:I17"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="A1:E37"/>
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -844,525 +1339,525 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>17</v>
+      <c r="A1" s="19" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="9" t="n">
+      <c r="A2" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="20" t="n">
         <v>80</v>
       </c>
-      <c r="C2" s="10" t="n">
+      <c r="C2" s="21" t="n">
         <v>60</v>
       </c>
-      <c r="D2" s="10" t="n">
+      <c r="D2" s="22" t="n">
         <f aca="false">IF(A2="","",B2*C2)</f>
         <v>4800</v>
       </c>
-      <c r="E2" s="11" t="n">
+      <c r="E2" s="23" t="n">
         <f aca="false">IFERROR(D2/$D$32,0)</f>
         <v>0.44423877834336</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="12" t="n">
+      <c r="A3" s="20" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="C3" s="13" t="n">
+      <c r="C3" s="21" t="n">
         <v>45</v>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="22" t="n">
         <f aca="false">IF(A3="","",B3*C3)</f>
         <v>1350</v>
       </c>
-      <c r="E3" s="14" t="n">
+      <c r="E3" s="23" t="n">
         <f aca="false">IFERROR(D3/$D$32,0)</f>
         <v>0.12494215640907</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="9" t="n">
+      <c r="A4" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="20" t="n">
         <v>40</v>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="21" t="n">
         <v>95</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="22" t="n">
         <f aca="false">IF(A4="","",B4*C4)</f>
         <v>3800</v>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="23" t="n">
         <f aca="false">IFERROR(D4/$D$32,0)</f>
         <v>0.35168903285516</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5" s="12" t="n">
+      <c r="A5" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="21" t="n">
         <v>25</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="22" t="n">
         <f aca="false">IF(A5="","",B5*C5)</f>
         <v>375</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="23" t="n">
         <f aca="false">IFERROR(D5/$D$32,0)</f>
         <v>0.034706154558075</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" s="9" t="n">
+      <c r="A6" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="22" t="n">
         <f aca="false">IF(A6="","",B6*C6)</f>
         <v>480</v>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="23" t="n">
         <f aca="false">IFERROR(D6/$D$32,0)</f>
         <v>0.044423877834336</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13" t="str">
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="22" t="str">
         <f aca="false">IF(A7="","",B7*C7)</f>
         <v/>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="23" t="n">
         <f aca="false">IFERROR(D7/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10" t="str">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+      <c r="C8" s="21"/>
+      <c r="D8" s="22" t="str">
         <f aca="false">IF(A8="","",B8*C8)</f>
         <v/>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="23" t="n">
         <f aca="false">IFERROR(D8/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12"/>
-      <c r="B9" s="12"/>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13" t="str">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="22" t="str">
         <f aca="false">IF(A9="","",B9*C9)</f>
         <v/>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="23" t="n">
         <f aca="false">IFERROR(D9/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10" t="str">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="22" t="str">
         <f aca="false">IF(A10="","",B10*C10)</f>
         <v/>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="23" t="n">
         <f aca="false">IFERROR(D10/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13" t="str">
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="22" t="str">
         <f aca="false">IF(A11="","",B11*C11)</f>
         <v/>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="23" t="n">
         <f aca="false">IFERROR(D11/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10" t="str">
+      <c r="A12" s="20"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="22" t="str">
         <f aca="false">IF(A12="","",B12*C12)</f>
         <v/>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="23" t="n">
         <f aca="false">IFERROR(D12/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13" t="str">
+      <c r="A13" s="20"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="22" t="str">
         <f aca="false">IF(A13="","",B13*C13)</f>
         <v/>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="23" t="n">
         <f aca="false">IFERROR(D13/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10" t="str">
+      <c r="A14" s="20"/>
+      <c r="B14" s="20"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="22" t="str">
         <f aca="false">IF(A14="","",B14*C14)</f>
         <v/>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="23" t="n">
         <f aca="false">IFERROR(D14/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13" t="str">
+      <c r="A15" s="20"/>
+      <c r="B15" s="20"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="22" t="str">
         <f aca="false">IF(A15="","",B15*C15)</f>
         <v/>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="23" t="n">
         <f aca="false">IFERROR(D15/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10" t="str">
+      <c r="A16" s="20"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="22" t="str">
         <f aca="false">IF(A16="","",B16*C16)</f>
         <v/>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="23" t="n">
         <f aca="false">IFERROR(D16/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="13" t="str">
+      <c r="A17" s="20"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="22" t="str">
         <f aca="false">IF(A17="","",B17*C17)</f>
         <v/>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="E17" s="23" t="n">
         <f aca="false">IFERROR(D17/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10" t="str">
+      <c r="A18" s="20"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="22" t="str">
         <f aca="false">IF(A18="","",B18*C18)</f>
         <v/>
       </c>
-      <c r="E18" s="11" t="n">
+      <c r="E18" s="23" t="n">
         <f aca="false">IFERROR(D18/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13" t="str">
+      <c r="A19" s="20"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="22" t="str">
         <f aca="false">IF(A19="","",B19*C19)</f>
         <v/>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="E19" s="23" t="n">
         <f aca="false">IFERROR(D19/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10" t="str">
+      <c r="A20" s="20"/>
+      <c r="B20" s="20"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="22" t="str">
         <f aca="false">IF(A20="","",B20*C20)</f>
         <v/>
       </c>
-      <c r="E20" s="11" t="n">
+      <c r="E20" s="23" t="n">
         <f aca="false">IFERROR(D20/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13" t="str">
+      <c r="A21" s="20"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="22" t="str">
         <f aca="false">IF(A21="","",B21*C21)</f>
         <v/>
       </c>
-      <c r="E21" s="14" t="n">
+      <c r="E21" s="23" t="n">
         <f aca="false">IFERROR(D21/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9"/>
-      <c r="B22" s="9"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10" t="str">
+      <c r="A22" s="20"/>
+      <c r="B22" s="20"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="22" t="str">
         <f aca="false">IF(A22="","",B22*C22)</f>
         <v/>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E22" s="23" t="n">
         <f aca="false">IFERROR(D22/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13" t="str">
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="22" t="str">
         <f aca="false">IF(A23="","",B23*C23)</f>
         <v/>
       </c>
-      <c r="E23" s="14" t="n">
+      <c r="E23" s="23" t="n">
         <f aca="false">IFERROR(D23/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10" t="str">
+      <c r="A24" s="20"/>
+      <c r="B24" s="20"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="22" t="str">
         <f aca="false">IF(A24="","",B24*C24)</f>
         <v/>
       </c>
-      <c r="E24" s="11" t="n">
+      <c r="E24" s="23" t="n">
         <f aca="false">IFERROR(D24/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="13" t="str">
+      <c r="A25" s="20"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="22" t="str">
         <f aca="false">IF(A25="","",B25*C25)</f>
         <v/>
       </c>
-      <c r="E25" s="14" t="n">
+      <c r="E25" s="23" t="n">
         <f aca="false">IFERROR(D25/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9"/>
-      <c r="B26" s="9"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10" t="str">
+      <c r="A26" s="20"/>
+      <c r="B26" s="20"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="22" t="str">
         <f aca="false">IF(A26="","",B26*C26)</f>
         <v/>
       </c>
-      <c r="E26" s="11" t="n">
+      <c r="E26" s="23" t="n">
         <f aca="false">IFERROR(D26/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13" t="str">
+      <c r="A27" s="20"/>
+      <c r="B27" s="20"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="22" t="str">
         <f aca="false">IF(A27="","",B27*C27)</f>
         <v/>
       </c>
-      <c r="E27" s="14" t="n">
+      <c r="E27" s="23" t="n">
         <f aca="false">IFERROR(D27/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10" t="str">
+      <c r="A28" s="20"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="22" t="str">
         <f aca="false">IF(A28="","",B28*C28)</f>
         <v/>
       </c>
-      <c r="E28" s="11" t="n">
+      <c r="E28" s="23" t="n">
         <f aca="false">IFERROR(D28/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="13"/>
-      <c r="D29" s="13" t="str">
+      <c r="A29" s="20"/>
+      <c r="B29" s="20"/>
+      <c r="C29" s="21"/>
+      <c r="D29" s="22" t="str">
         <f aca="false">IF(A29="","",B29*C29)</f>
         <v/>
       </c>
-      <c r="E29" s="14" t="n">
+      <c r="E29" s="23" t="n">
         <f aca="false">IFERROR(D29/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="9"/>
-      <c r="B30" s="9"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10" t="str">
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="22" t="str">
         <f aca="false">IF(A30="","",B30*C30)</f>
         <v/>
       </c>
-      <c r="E30" s="11" t="n">
+      <c r="E30" s="23" t="n">
         <f aca="false">IFERROR(D30/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="13" t="str">
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="22" t="str">
         <f aca="false">IF(A31="","",B31*C31)</f>
         <v/>
       </c>
-      <c r="E31" s="14" t="n">
+      <c r="E31" s="23" t="n">
         <f aca="false">IFERROR(D31/$D$32,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B32" s="8" t="n">
+      <c r="A32" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B32" s="19" t="n">
         <f aca="false">SUM(B2:B31)</f>
         <v>177</v>
       </c>
-      <c r="C32" s="15"/>
-      <c r="D32" s="15" t="n">
+      <c r="C32" s="24"/>
+      <c r="D32" s="24" t="n">
         <f aca="false">SUM(D2:D31)</f>
         <v>10805</v>
       </c>
-      <c r="E32" s="16" t="n">
+      <c r="E32" s="25" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B33" s="12" t="n">
+      <c r="A33" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B33" s="20" t="n">
         <v>140</v>
       </c>
-      <c r="C33" s="13"/>
-      <c r="D33" s="13"/>
-      <c r="E33" s="12" t="s">
-        <v>25</v>
+      <c r="C33" s="26"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="27" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="B34" s="17"/>
-      <c r="C34" s="18"/>
-      <c r="D34" s="18" t="n">
+      <c r="A34" s="28" t="s">
+        <v>51</v>
+      </c>
+      <c r="B34" s="28"/>
+      <c r="C34" s="29"/>
+      <c r="D34" s="29" t="n">
         <f aca="false">IFERROR(D32/B33,0)</f>
         <v>77.1785714285714</v>
       </c>
-      <c r="E34" s="17" t="s">
-        <v>27</v>
+      <c r="E34" s="28" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="B35" s="17"/>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18" t="n">
+      <c r="A35" s="28" t="s">
+        <v>53</v>
+      </c>
+      <c r="B35" s="28"/>
+      <c r="C35" s="29"/>
+      <c r="D35" s="29" t="n">
         <v>75</v>
       </c>
-      <c r="E35" s="17" t="s">
-        <v>25</v>
+      <c r="E35" s="28" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="17" t="s">
-        <v>29</v>
-      </c>
-      <c r="B36" s="17"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18" t="n">
+      <c r="A36" s="28" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="28"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29" t="n">
         <f aca="false">D35-D34</f>
         <v>-2.17857142857143</v>
       </c>
-      <c r="E36" s="17" t="s">
-        <v>30</v>
+      <c r="E36" s="28" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="B37" s="17"/>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18" t="n">
+      <c r="A37" s="28" t="s">
+        <v>56</v>
+      </c>
+      <c r="B37" s="28"/>
+      <c r="C37" s="29"/>
+      <c r="D37" s="29" t="n">
         <f aca="false">B33*D35</f>
         <v>10500</v>
       </c>
-      <c r="E37" s="17" t="s">
-        <v>32</v>
+      <c r="E37" s="28" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>